<commit_message>
Update GAA results for 2026-10-25
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2338"/>
+  <dimension ref="A1:G2339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83314,6 +83314,43 @@
         </is>
       </c>
     </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr">
+        <is>
+          <t>Shinty-Hurling International</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="D2339" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="E2339" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh, Cork</t>
+        </is>
+      </c>
+      <c r="F2339" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2339" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>